<commit_message>
Ajuste de sección predeterminada a Dashboard y mantenimiento de persistencia en recarga de página.
</commit_message>
<xml_diff>
--- a/public/Formato_de_Carga_de_Asistencia.xlsx
+++ b/public/Formato_de_Carga_de_Asistencia.xlsx
@@ -508,7 +508,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L200"/>
+  <dimension ref="A1:L427"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="13.9" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.28515625" bestFit="1" customWidth="1"/>
@@ -579,7 +579,10 @@
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
-      <c r="K3" s="6"/>
+      <c r="K3" s="6" t="str">
+        <f>IF(A3="","",SUM(D3:J3))</f>
+        <v/>
+      </c>
       <c r="L3" s="1"/>
     </row>
     <row r="4" spans="1:12" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -593,7 +596,10 @@
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
       <c r="J4" s="5"/>
-      <c r="K4" s="6"/>
+      <c r="K4" s="6" t="str">
+        <f t="shared" ref="K4:K67" si="0">IF(A4="","",SUM(D4:J4))</f>
+        <v/>
+      </c>
       <c r="L4" s="1"/>
     </row>
     <row r="5" spans="1:12" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -607,7 +613,10 @@
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
-      <c r="K5" s="6"/>
+      <c r="K5" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="L5" s="1"/>
     </row>
     <row r="6" spans="1:12" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -621,7 +630,10 @@
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
-      <c r="K6" s="6"/>
+      <c r="K6" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="L6" s="1"/>
     </row>
     <row r="7" spans="1:12" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -635,7 +647,10 @@
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
       <c r="J7" s="5"/>
-      <c r="K7" s="6"/>
+      <c r="K7" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="L7" s="1"/>
     </row>
     <row r="8" spans="1:12" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -649,7 +664,10 @@
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
-      <c r="K8" s="6"/>
+      <c r="K8" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="L8" s="1"/>
     </row>
     <row r="9" spans="1:12" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -663,7 +681,10 @@
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
-      <c r="K9" s="6"/>
+      <c r="K9" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="L9" s="1"/>
     </row>
     <row r="10" spans="1:12" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -677,7 +698,10 @@
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
-      <c r="K10" s="6"/>
+      <c r="K10" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="L10" s="1"/>
     </row>
     <row r="11" spans="1:12" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -691,7 +715,10 @@
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
-      <c r="K11" s="6"/>
+      <c r="K11" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="12" spans="1:12" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
@@ -704,7 +731,10 @@
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
-      <c r="K12" s="6"/>
+      <c r="K12" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="13" spans="1:12" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
@@ -717,7 +747,10 @@
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
-      <c r="K13" s="6"/>
+      <c r="K13" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="14" spans="1:12" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
@@ -730,7 +763,10 @@
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
-      <c r="K14" s="6"/>
+      <c r="K14" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="15" spans="1:12" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
@@ -743,7 +779,10 @@
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
-      <c r="K15" s="6"/>
+      <c r="K15" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="16" spans="1:12" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8"/>
@@ -756,7 +795,10 @@
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>
       <c r="J16" s="5"/>
-      <c r="K16" s="6"/>
+      <c r="K16" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="17" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
@@ -769,7 +811,10 @@
       <c r="H17" s="5"/>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
-      <c r="K17" s="6"/>
+      <c r="K17" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="18" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
@@ -782,7 +827,10 @@
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
       <c r="J18" s="5"/>
-      <c r="K18" s="6"/>
+      <c r="K18" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="19" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8"/>
@@ -795,7 +843,10 @@
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
-      <c r="K19" s="6"/>
+      <c r="K19" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="20" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8"/>
@@ -808,7 +859,10 @@
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
-      <c r="K20" s="6"/>
+      <c r="K20" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="21" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
@@ -821,7 +875,10 @@
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
-      <c r="K21" s="6"/>
+      <c r="K21" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="22" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
@@ -834,7 +891,10 @@
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
       <c r="J22" s="5"/>
-      <c r="K22" s="6"/>
+      <c r="K22" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="23" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="10"/>
@@ -847,7 +907,10 @@
       <c r="H23" s="7"/>
       <c r="I23" s="7"/>
       <c r="J23" s="7"/>
-      <c r="K23" s="7"/>
+      <c r="K23" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="24" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="10"/>
@@ -860,7 +923,10 @@
       <c r="H24" s="7"/>
       <c r="I24" s="7"/>
       <c r="J24" s="7"/>
-      <c r="K24" s="7"/>
+      <c r="K24" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="25" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="10"/>
@@ -873,7 +939,10 @@
       <c r="H25" s="7"/>
       <c r="I25" s="7"/>
       <c r="J25" s="7"/>
-      <c r="K25" s="7"/>
+      <c r="K25" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="26" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="10"/>
@@ -886,7 +955,10 @@
       <c r="H26" s="7"/>
       <c r="I26" s="7"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
+      <c r="K26" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="27" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="10"/>
@@ -899,7 +971,10 @@
       <c r="H27" s="7"/>
       <c r="I27" s="7"/>
       <c r="J27" s="7"/>
-      <c r="K27" s="7"/>
+      <c r="K27" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="28" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="10"/>
@@ -912,7 +987,10 @@
       <c r="H28" s="7"/>
       <c r="I28" s="7"/>
       <c r="J28" s="7"/>
-      <c r="K28" s="7"/>
+      <c r="K28" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="29" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10"/>
@@ -925,7 +1003,10 @@
       <c r="H29" s="7"/>
       <c r="I29" s="7"/>
       <c r="J29" s="7"/>
-      <c r="K29" s="7"/>
+      <c r="K29" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="30" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="10"/>
@@ -938,7 +1019,10 @@
       <c r="H30" s="7"/>
       <c r="I30" s="7"/>
       <c r="J30" s="7"/>
-      <c r="K30" s="7"/>
+      <c r="K30" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="31" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
@@ -951,7 +1035,10 @@
       <c r="H31" s="7"/>
       <c r="I31" s="7"/>
       <c r="J31" s="7"/>
-      <c r="K31" s="7"/>
+      <c r="K31" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="32" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="10"/>
@@ -964,7 +1051,10 @@
       <c r="H32" s="7"/>
       <c r="I32" s="7"/>
       <c r="J32" s="7"/>
-      <c r="K32" s="7"/>
+      <c r="K32" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="33" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="10"/>
@@ -977,7 +1067,10 @@
       <c r="H33" s="7"/>
       <c r="I33" s="7"/>
       <c r="J33" s="7"/>
-      <c r="K33" s="7"/>
+      <c r="K33" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="34" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="10"/>
@@ -990,7 +1083,10 @@
       <c r="H34" s="7"/>
       <c r="I34" s="7"/>
       <c r="J34" s="7"/>
-      <c r="K34" s="7"/>
+      <c r="K34" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="35" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="10"/>
@@ -1003,7 +1099,10 @@
       <c r="H35" s="7"/>
       <c r="I35" s="7"/>
       <c r="J35" s="7"/>
-      <c r="K35" s="7"/>
+      <c r="K35" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="36" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="10"/>
@@ -1016,7 +1115,10 @@
       <c r="H36" s="7"/>
       <c r="I36" s="7"/>
       <c r="J36" s="7"/>
-      <c r="K36" s="7"/>
+      <c r="K36" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="37" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="10"/>
@@ -1029,7 +1131,10 @@
       <c r="H37" s="7"/>
       <c r="I37" s="7"/>
       <c r="J37" s="7"/>
-      <c r="K37" s="7"/>
+      <c r="K37" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="38" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="10"/>
@@ -1042,7 +1147,10 @@
       <c r="H38" s="7"/>
       <c r="I38" s="7"/>
       <c r="J38" s="7"/>
-      <c r="K38" s="7"/>
+      <c r="K38" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="39" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="10"/>
@@ -1055,7 +1163,10 @@
       <c r="H39" s="7"/>
       <c r="I39" s="7"/>
       <c r="J39" s="7"/>
-      <c r="K39" s="7"/>
+      <c r="K39" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="40" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="10"/>
@@ -1068,7 +1179,10 @@
       <c r="H40" s="7"/>
       <c r="I40" s="7"/>
       <c r="J40" s="7"/>
-      <c r="K40" s="7"/>
+      <c r="K40" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="41" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="10"/>
@@ -1081,7 +1195,10 @@
       <c r="H41" s="7"/>
       <c r="I41" s="7"/>
       <c r="J41" s="7"/>
-      <c r="K41" s="7"/>
+      <c r="K41" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="42" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="10"/>
@@ -1094,7 +1211,10 @@
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
       <c r="J42" s="7"/>
-      <c r="K42" s="7"/>
+      <c r="K42" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="43" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="10"/>
@@ -1107,7 +1227,10 @@
       <c r="H43" s="7"/>
       <c r="I43" s="7"/>
       <c r="J43" s="7"/>
-      <c r="K43" s="7"/>
+      <c r="K43" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="44" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="10"/>
@@ -1120,7 +1243,10 @@
       <c r="H44" s="7"/>
       <c r="I44" s="7"/>
       <c r="J44" s="7"/>
-      <c r="K44" s="7"/>
+      <c r="K44" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="45" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="10"/>
@@ -1133,7 +1259,10 @@
       <c r="H45" s="7"/>
       <c r="I45" s="7"/>
       <c r="J45" s="7"/>
-      <c r="K45" s="7"/>
+      <c r="K45" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="46" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="10"/>
@@ -1146,7 +1275,10 @@
       <c r="H46" s="7"/>
       <c r="I46" s="7"/>
       <c r="J46" s="7"/>
-      <c r="K46" s="7"/>
+      <c r="K46" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="47" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="10"/>
@@ -1159,7 +1291,10 @@
       <c r="H47" s="7"/>
       <c r="I47" s="7"/>
       <c r="J47" s="7"/>
-      <c r="K47" s="7"/>
+      <c r="K47" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="48" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="10"/>
@@ -1172,7 +1307,10 @@
       <c r="H48" s="7"/>
       <c r="I48" s="7"/>
       <c r="J48" s="7"/>
-      <c r="K48" s="7"/>
+      <c r="K48" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="49" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="10"/>
@@ -1185,7 +1323,10 @@
       <c r="H49" s="7"/>
       <c r="I49" s="7"/>
       <c r="J49" s="7"/>
-      <c r="K49" s="7"/>
+      <c r="K49" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="50" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="10"/>
@@ -1198,7 +1339,10 @@
       <c r="H50" s="7"/>
       <c r="I50" s="7"/>
       <c r="J50" s="7"/>
-      <c r="K50" s="7"/>
+      <c r="K50" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="51" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="10"/>
@@ -1211,7 +1355,10 @@
       <c r="H51" s="7"/>
       <c r="I51" s="7"/>
       <c r="J51" s="7"/>
-      <c r="K51" s="7"/>
+      <c r="K51" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="52" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="10"/>
@@ -1224,7 +1371,10 @@
       <c r="H52" s="7"/>
       <c r="I52" s="7"/>
       <c r="J52" s="7"/>
-      <c r="K52" s="7"/>
+      <c r="K52" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="53" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="10"/>
@@ -1237,7 +1387,10 @@
       <c r="H53" s="7"/>
       <c r="I53" s="7"/>
       <c r="J53" s="7"/>
-      <c r="K53" s="7"/>
+      <c r="K53" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="54" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="10"/>
@@ -1250,7 +1403,10 @@
       <c r="H54" s="7"/>
       <c r="I54" s="7"/>
       <c r="J54" s="7"/>
-      <c r="K54" s="7"/>
+      <c r="K54" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="55" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="10"/>
@@ -1263,7 +1419,10 @@
       <c r="H55" s="7"/>
       <c r="I55" s="7"/>
       <c r="J55" s="7"/>
-      <c r="K55" s="7"/>
+      <c r="K55" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="56" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="10"/>
@@ -1276,7 +1435,10 @@
       <c r="H56" s="7"/>
       <c r="I56" s="7"/>
       <c r="J56" s="7"/>
-      <c r="K56" s="7"/>
+      <c r="K56" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="57" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="10"/>
@@ -1289,7 +1451,10 @@
       <c r="H57" s="7"/>
       <c r="I57" s="7"/>
       <c r="J57" s="7"/>
-      <c r="K57" s="7"/>
+      <c r="K57" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="58" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="10"/>
@@ -1302,7 +1467,10 @@
       <c r="H58" s="7"/>
       <c r="I58" s="7"/>
       <c r="J58" s="7"/>
-      <c r="K58" s="7"/>
+      <c r="K58" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="59" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="10"/>
@@ -1315,7 +1483,10 @@
       <c r="H59" s="7"/>
       <c r="I59" s="7"/>
       <c r="J59" s="7"/>
-      <c r="K59" s="7"/>
+      <c r="K59" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="60" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="10"/>
@@ -1328,7 +1499,10 @@
       <c r="H60" s="7"/>
       <c r="I60" s="7"/>
       <c r="J60" s="7"/>
-      <c r="K60" s="7"/>
+      <c r="K60" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="61" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="10"/>
@@ -1341,7 +1515,10 @@
       <c r="H61" s="7"/>
       <c r="I61" s="7"/>
       <c r="J61" s="7"/>
-      <c r="K61" s="7"/>
+      <c r="K61" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="62" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="10"/>
@@ -1354,7 +1531,10 @@
       <c r="H62" s="7"/>
       <c r="I62" s="7"/>
       <c r="J62" s="7"/>
-      <c r="K62" s="7"/>
+      <c r="K62" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="63" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="10"/>
@@ -1367,7 +1547,10 @@
       <c r="H63" s="7"/>
       <c r="I63" s="7"/>
       <c r="J63" s="7"/>
-      <c r="K63" s="7"/>
+      <c r="K63" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="64" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="10"/>
@@ -1380,7 +1563,10 @@
       <c r="H64" s="7"/>
       <c r="I64" s="7"/>
       <c r="J64" s="7"/>
-      <c r="K64" s="7"/>
+      <c r="K64" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="65" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="10"/>
@@ -1393,7 +1579,10 @@
       <c r="H65" s="7"/>
       <c r="I65" s="7"/>
       <c r="J65" s="7"/>
-      <c r="K65" s="7"/>
+      <c r="K65" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="66" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="10"/>
@@ -1406,7 +1595,10 @@
       <c r="H66" s="7"/>
       <c r="I66" s="7"/>
       <c r="J66" s="7"/>
-      <c r="K66" s="7"/>
+      <c r="K66" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="67" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="10"/>
@@ -1419,7 +1611,10 @@
       <c r="H67" s="7"/>
       <c r="I67" s="7"/>
       <c r="J67" s="7"/>
-      <c r="K67" s="7"/>
+      <c r="K67" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
     </row>
     <row r="68" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="10"/>
@@ -1432,7 +1627,10 @@
       <c r="H68" s="7"/>
       <c r="I68" s="7"/>
       <c r="J68" s="7"/>
-      <c r="K68" s="7"/>
+      <c r="K68" s="6" t="str">
+        <f t="shared" ref="K68:K131" si="1">IF(A68="","",SUM(D68:J68))</f>
+        <v/>
+      </c>
     </row>
     <row r="69" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="10"/>
@@ -1445,7 +1643,10 @@
       <c r="H69" s="7"/>
       <c r="I69" s="7"/>
       <c r="J69" s="7"/>
-      <c r="K69" s="7"/>
+      <c r="K69" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="70" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="10"/>
@@ -1458,7 +1659,10 @@
       <c r="H70" s="7"/>
       <c r="I70" s="7"/>
       <c r="J70" s="7"/>
-      <c r="K70" s="7"/>
+      <c r="K70" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="71" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="10"/>
@@ -1471,7 +1675,10 @@
       <c r="H71" s="7"/>
       <c r="I71" s="7"/>
       <c r="J71" s="7"/>
-      <c r="K71" s="7"/>
+      <c r="K71" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="72" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="10"/>
@@ -1484,7 +1691,10 @@
       <c r="H72" s="7"/>
       <c r="I72" s="7"/>
       <c r="J72" s="7"/>
-      <c r="K72" s="7"/>
+      <c r="K72" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="73" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="10"/>
@@ -1497,7 +1707,10 @@
       <c r="H73" s="7"/>
       <c r="I73" s="7"/>
       <c r="J73" s="7"/>
-      <c r="K73" s="7"/>
+      <c r="K73" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="74" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="10"/>
@@ -1510,7 +1723,10 @@
       <c r="H74" s="7"/>
       <c r="I74" s="7"/>
       <c r="J74" s="7"/>
-      <c r="K74" s="7"/>
+      <c r="K74" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="75" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="10"/>
@@ -1523,7 +1739,10 @@
       <c r="H75" s="7"/>
       <c r="I75" s="7"/>
       <c r="J75" s="7"/>
-      <c r="K75" s="7"/>
+      <c r="K75" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="76" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="10"/>
@@ -1536,7 +1755,10 @@
       <c r="H76" s="7"/>
       <c r="I76" s="7"/>
       <c r="J76" s="7"/>
-      <c r="K76" s="7"/>
+      <c r="K76" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="77" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="10"/>
@@ -1549,7 +1771,10 @@
       <c r="H77" s="7"/>
       <c r="I77" s="7"/>
       <c r="J77" s="7"/>
-      <c r="K77" s="7"/>
+      <c r="K77" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="78" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="10"/>
@@ -1562,7 +1787,10 @@
       <c r="H78" s="7"/>
       <c r="I78" s="7"/>
       <c r="J78" s="7"/>
-      <c r="K78" s="7"/>
+      <c r="K78" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="79" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="10"/>
@@ -1575,7 +1803,10 @@
       <c r="H79" s="7"/>
       <c r="I79" s="7"/>
       <c r="J79" s="7"/>
-      <c r="K79" s="7"/>
+      <c r="K79" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="80" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="10"/>
@@ -1588,7 +1819,10 @@
       <c r="H80" s="7"/>
       <c r="I80" s="7"/>
       <c r="J80" s="7"/>
-      <c r="K80" s="7"/>
+      <c r="K80" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="81" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="10"/>
@@ -1601,7 +1835,10 @@
       <c r="H81" s="7"/>
       <c r="I81" s="7"/>
       <c r="J81" s="7"/>
-      <c r="K81" s="7"/>
+      <c r="K81" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="82" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="10"/>
@@ -1614,7 +1851,10 @@
       <c r="H82" s="7"/>
       <c r="I82" s="7"/>
       <c r="J82" s="7"/>
-      <c r="K82" s="7"/>
+      <c r="K82" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="83" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="10"/>
@@ -1627,7 +1867,10 @@
       <c r="H83" s="7"/>
       <c r="I83" s="7"/>
       <c r="J83" s="7"/>
-      <c r="K83" s="7"/>
+      <c r="K83" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="84" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="10"/>
@@ -1640,7 +1883,10 @@
       <c r="H84" s="7"/>
       <c r="I84" s="7"/>
       <c r="J84" s="7"/>
-      <c r="K84" s="7"/>
+      <c r="K84" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="85" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="10"/>
@@ -1653,7 +1899,10 @@
       <c r="H85" s="7"/>
       <c r="I85" s="7"/>
       <c r="J85" s="7"/>
-      <c r="K85" s="7"/>
+      <c r="K85" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="86" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="10"/>
@@ -1666,7 +1915,10 @@
       <c r="H86" s="7"/>
       <c r="I86" s="7"/>
       <c r="J86" s="7"/>
-      <c r="K86" s="7"/>
+      <c r="K86" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="87" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="10"/>
@@ -1679,7 +1931,10 @@
       <c r="H87" s="7"/>
       <c r="I87" s="7"/>
       <c r="J87" s="7"/>
-      <c r="K87" s="7"/>
+      <c r="K87" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="88" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="10"/>
@@ -1692,7 +1947,10 @@
       <c r="H88" s="7"/>
       <c r="I88" s="7"/>
       <c r="J88" s="7"/>
-      <c r="K88" s="7"/>
+      <c r="K88" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="89" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="10"/>
@@ -1705,7 +1963,10 @@
       <c r="H89" s="7"/>
       <c r="I89" s="7"/>
       <c r="J89" s="7"/>
-      <c r="K89" s="7"/>
+      <c r="K89" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="90" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="10"/>
@@ -1718,7 +1979,10 @@
       <c r="H90" s="7"/>
       <c r="I90" s="7"/>
       <c r="J90" s="7"/>
-      <c r="K90" s="7"/>
+      <c r="K90" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="91" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="10"/>
@@ -1731,7 +1995,10 @@
       <c r="H91" s="7"/>
       <c r="I91" s="7"/>
       <c r="J91" s="7"/>
-      <c r="K91" s="7"/>
+      <c r="K91" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="92" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="10"/>
@@ -1744,7 +2011,10 @@
       <c r="H92" s="7"/>
       <c r="I92" s="7"/>
       <c r="J92" s="7"/>
-      <c r="K92" s="7"/>
+      <c r="K92" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="93" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="10"/>
@@ -1757,7 +2027,10 @@
       <c r="H93" s="7"/>
       <c r="I93" s="7"/>
       <c r="J93" s="7"/>
-      <c r="K93" s="7"/>
+      <c r="K93" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="94" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="10"/>
@@ -1770,7 +2043,10 @@
       <c r="H94" s="7"/>
       <c r="I94" s="7"/>
       <c r="J94" s="7"/>
-      <c r="K94" s="7"/>
+      <c r="K94" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="95" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="10"/>
@@ -1783,7 +2059,10 @@
       <c r="H95" s="7"/>
       <c r="I95" s="7"/>
       <c r="J95" s="7"/>
-      <c r="K95" s="7"/>
+      <c r="K95" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="96" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="10"/>
@@ -1796,7 +2075,10 @@
       <c r="H96" s="7"/>
       <c r="I96" s="7"/>
       <c r="J96" s="7"/>
-      <c r="K96" s="7"/>
+      <c r="K96" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="97" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="10"/>
@@ -1809,7 +2091,10 @@
       <c r="H97" s="7"/>
       <c r="I97" s="7"/>
       <c r="J97" s="7"/>
-      <c r="K97" s="7"/>
+      <c r="K97" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="98" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="10"/>
@@ -1822,7 +2107,10 @@
       <c r="H98" s="7"/>
       <c r="I98" s="7"/>
       <c r="J98" s="7"/>
-      <c r="K98" s="7"/>
+      <c r="K98" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="99" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="10"/>
@@ -1835,7 +2123,10 @@
       <c r="H99" s="7"/>
       <c r="I99" s="7"/>
       <c r="J99" s="7"/>
-      <c r="K99" s="7"/>
+      <c r="K99" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="100" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="10"/>
@@ -1848,7 +2139,10 @@
       <c r="H100" s="7"/>
       <c r="I100" s="7"/>
       <c r="J100" s="7"/>
-      <c r="K100" s="7"/>
+      <c r="K100" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="101" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="10"/>
@@ -1861,7 +2155,10 @@
       <c r="H101" s="7"/>
       <c r="I101" s="7"/>
       <c r="J101" s="7"/>
-      <c r="K101" s="7"/>
+      <c r="K101" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="102" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="10"/>
@@ -1874,7 +2171,10 @@
       <c r="H102" s="7"/>
       <c r="I102" s="7"/>
       <c r="J102" s="7"/>
-      <c r="K102" s="7"/>
+      <c r="K102" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="103" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="10"/>
@@ -1887,7 +2187,10 @@
       <c r="H103" s="7"/>
       <c r="I103" s="7"/>
       <c r="J103" s="7"/>
-      <c r="K103" s="7"/>
+      <c r="K103" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="104" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="10"/>
@@ -1900,7 +2203,10 @@
       <c r="H104" s="7"/>
       <c r="I104" s="7"/>
       <c r="J104" s="7"/>
-      <c r="K104" s="7"/>
+      <c r="K104" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="105" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="10"/>
@@ -1913,7 +2219,10 @@
       <c r="H105" s="7"/>
       <c r="I105" s="7"/>
       <c r="J105" s="7"/>
-      <c r="K105" s="7"/>
+      <c r="K105" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="106" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="10"/>
@@ -1926,7 +2235,10 @@
       <c r="H106" s="7"/>
       <c r="I106" s="7"/>
       <c r="J106" s="7"/>
-      <c r="K106" s="7"/>
+      <c r="K106" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="107" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="10"/>
@@ -1939,7 +2251,10 @@
       <c r="H107" s="7"/>
       <c r="I107" s="7"/>
       <c r="J107" s="7"/>
-      <c r="K107" s="7"/>
+      <c r="K107" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="108" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="10"/>
@@ -1952,7 +2267,10 @@
       <c r="H108" s="7"/>
       <c r="I108" s="7"/>
       <c r="J108" s="7"/>
-      <c r="K108" s="7"/>
+      <c r="K108" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="109" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="10"/>
@@ -1965,7 +2283,10 @@
       <c r="H109" s="7"/>
       <c r="I109" s="7"/>
       <c r="J109" s="7"/>
-      <c r="K109" s="7"/>
+      <c r="K109" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="110" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="10"/>
@@ -1978,7 +2299,10 @@
       <c r="H110" s="7"/>
       <c r="I110" s="7"/>
       <c r="J110" s="7"/>
-      <c r="K110" s="7"/>
+      <c r="K110" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="111" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="10"/>
@@ -1991,7 +2315,10 @@
       <c r="H111" s="7"/>
       <c r="I111" s="7"/>
       <c r="J111" s="7"/>
-      <c r="K111" s="7"/>
+      <c r="K111" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="112" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="10"/>
@@ -2004,7 +2331,10 @@
       <c r="H112" s="7"/>
       <c r="I112" s="7"/>
       <c r="J112" s="7"/>
-      <c r="K112" s="7"/>
+      <c r="K112" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="113" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="10"/>
@@ -2017,7 +2347,10 @@
       <c r="H113" s="7"/>
       <c r="I113" s="7"/>
       <c r="J113" s="7"/>
-      <c r="K113" s="7"/>
+      <c r="K113" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="114" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="10"/>
@@ -2030,7 +2363,10 @@
       <c r="H114" s="7"/>
       <c r="I114" s="7"/>
       <c r="J114" s="7"/>
-      <c r="K114" s="7"/>
+      <c r="K114" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="115" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="10"/>
@@ -2043,7 +2379,10 @@
       <c r="H115" s="7"/>
       <c r="I115" s="7"/>
       <c r="J115" s="7"/>
-      <c r="K115" s="7"/>
+      <c r="K115" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="116" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="10"/>
@@ -2056,7 +2395,10 @@
       <c r="H116" s="7"/>
       <c r="I116" s="7"/>
       <c r="J116" s="7"/>
-      <c r="K116" s="7"/>
+      <c r="K116" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="117" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="10"/>
@@ -2069,7 +2411,10 @@
       <c r="H117" s="7"/>
       <c r="I117" s="7"/>
       <c r="J117" s="7"/>
-      <c r="K117" s="7"/>
+      <c r="K117" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="118" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="10"/>
@@ -2082,7 +2427,10 @@
       <c r="H118" s="7"/>
       <c r="I118" s="7"/>
       <c r="J118" s="7"/>
-      <c r="K118" s="7"/>
+      <c r="K118" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="119" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="10"/>
@@ -2095,7 +2443,10 @@
       <c r="H119" s="7"/>
       <c r="I119" s="7"/>
       <c r="J119" s="7"/>
-      <c r="K119" s="7"/>
+      <c r="K119" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="120" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="10"/>
@@ -2108,7 +2459,10 @@
       <c r="H120" s="7"/>
       <c r="I120" s="7"/>
       <c r="J120" s="7"/>
-      <c r="K120" s="7"/>
+      <c r="K120" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="121" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="10"/>
@@ -2121,7 +2475,10 @@
       <c r="H121" s="7"/>
       <c r="I121" s="7"/>
       <c r="J121" s="7"/>
-      <c r="K121" s="7"/>
+      <c r="K121" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="122" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="10"/>
@@ -2134,7 +2491,10 @@
       <c r="H122" s="7"/>
       <c r="I122" s="7"/>
       <c r="J122" s="7"/>
-      <c r="K122" s="7"/>
+      <c r="K122" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="123" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="10"/>
@@ -2147,7 +2507,10 @@
       <c r="H123" s="7"/>
       <c r="I123" s="7"/>
       <c r="J123" s="7"/>
-      <c r="K123" s="7"/>
+      <c r="K123" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="124" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="10"/>
@@ -2160,7 +2523,10 @@
       <c r="H124" s="7"/>
       <c r="I124" s="7"/>
       <c r="J124" s="7"/>
-      <c r="K124" s="7"/>
+      <c r="K124" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="125" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="10"/>
@@ -2173,7 +2539,10 @@
       <c r="H125" s="7"/>
       <c r="I125" s="7"/>
       <c r="J125" s="7"/>
-      <c r="K125" s="7"/>
+      <c r="K125" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="126" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="10"/>
@@ -2186,7 +2555,10 @@
       <c r="H126" s="7"/>
       <c r="I126" s="7"/>
       <c r="J126" s="7"/>
-      <c r="K126" s="7"/>
+      <c r="K126" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="127" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="10"/>
@@ -2199,7 +2571,10 @@
       <c r="H127" s="7"/>
       <c r="I127" s="7"/>
       <c r="J127" s="7"/>
-      <c r="K127" s="7"/>
+      <c r="K127" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="128" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="10"/>
@@ -2212,7 +2587,10 @@
       <c r="H128" s="7"/>
       <c r="I128" s="7"/>
       <c r="J128" s="7"/>
-      <c r="K128" s="7"/>
+      <c r="K128" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="129" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="10"/>
@@ -2225,7 +2603,10 @@
       <c r="H129" s="7"/>
       <c r="I129" s="7"/>
       <c r="J129" s="7"/>
-      <c r="K129" s="7"/>
+      <c r="K129" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="130" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="10"/>
@@ -2238,7 +2619,10 @@
       <c r="H130" s="7"/>
       <c r="I130" s="7"/>
       <c r="J130" s="7"/>
-      <c r="K130" s="7"/>
+      <c r="K130" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="131" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="10"/>
@@ -2251,7 +2635,10 @@
       <c r="H131" s="7"/>
       <c r="I131" s="7"/>
       <c r="J131" s="7"/>
-      <c r="K131" s="7"/>
+      <c r="K131" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
     </row>
     <row r="132" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="10"/>
@@ -2264,7 +2651,10 @@
       <c r="H132" s="7"/>
       <c r="I132" s="7"/>
       <c r="J132" s="7"/>
-      <c r="K132" s="7"/>
+      <c r="K132" s="6" t="str">
+        <f t="shared" ref="K132:K195" si="2">IF(A132="","",SUM(D132:J132))</f>
+        <v/>
+      </c>
     </row>
     <row r="133" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="10"/>
@@ -2277,7 +2667,10 @@
       <c r="H133" s="7"/>
       <c r="I133" s="7"/>
       <c r="J133" s="7"/>
-      <c r="K133" s="7"/>
+      <c r="K133" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="134" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="10"/>
@@ -2290,7 +2683,10 @@
       <c r="H134" s="7"/>
       <c r="I134" s="7"/>
       <c r="J134" s="7"/>
-      <c r="K134" s="7"/>
+      <c r="K134" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="135" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="10"/>
@@ -2303,7 +2699,10 @@
       <c r="H135" s="7"/>
       <c r="I135" s="7"/>
       <c r="J135" s="7"/>
-      <c r="K135" s="7"/>
+      <c r="K135" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="136" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="10"/>
@@ -2316,7 +2715,10 @@
       <c r="H136" s="7"/>
       <c r="I136" s="7"/>
       <c r="J136" s="7"/>
-      <c r="K136" s="7"/>
+      <c r="K136" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="137" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="10"/>
@@ -2329,7 +2731,10 @@
       <c r="H137" s="7"/>
       <c r="I137" s="7"/>
       <c r="J137" s="7"/>
-      <c r="K137" s="7"/>
+      <c r="K137" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="138" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="10"/>
@@ -2342,7 +2747,10 @@
       <c r="H138" s="7"/>
       <c r="I138" s="7"/>
       <c r="J138" s="7"/>
-      <c r="K138" s="7"/>
+      <c r="K138" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="139" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="10"/>
@@ -2355,7 +2763,10 @@
       <c r="H139" s="7"/>
       <c r="I139" s="7"/>
       <c r="J139" s="7"/>
-      <c r="K139" s="7"/>
+      <c r="K139" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="140" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="10"/>
@@ -2368,7 +2779,10 @@
       <c r="H140" s="7"/>
       <c r="I140" s="7"/>
       <c r="J140" s="7"/>
-      <c r="K140" s="7"/>
+      <c r="K140" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="141" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="10"/>
@@ -2381,7 +2795,10 @@
       <c r="H141" s="7"/>
       <c r="I141" s="7"/>
       <c r="J141" s="7"/>
-      <c r="K141" s="7"/>
+      <c r="K141" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="142" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="10"/>
@@ -2394,7 +2811,10 @@
       <c r="H142" s="7"/>
       <c r="I142" s="7"/>
       <c r="J142" s="7"/>
-      <c r="K142" s="7"/>
+      <c r="K142" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="143" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="10"/>
@@ -2407,7 +2827,10 @@
       <c r="H143" s="7"/>
       <c r="I143" s="7"/>
       <c r="J143" s="7"/>
-      <c r="K143" s="7"/>
+      <c r="K143" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="144" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="10"/>
@@ -2420,7 +2843,10 @@
       <c r="H144" s="7"/>
       <c r="I144" s="7"/>
       <c r="J144" s="7"/>
-      <c r="K144" s="7"/>
+      <c r="K144" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="145" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="10"/>
@@ -2433,7 +2859,10 @@
       <c r="H145" s="7"/>
       <c r="I145" s="7"/>
       <c r="J145" s="7"/>
-      <c r="K145" s="7"/>
+      <c r="K145" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="146" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="10"/>
@@ -2446,7 +2875,10 @@
       <c r="H146" s="7"/>
       <c r="I146" s="7"/>
       <c r="J146" s="7"/>
-      <c r="K146" s="7"/>
+      <c r="K146" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="147" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="10"/>
@@ -2459,7 +2891,10 @@
       <c r="H147" s="7"/>
       <c r="I147" s="7"/>
       <c r="J147" s="7"/>
-      <c r="K147" s="7"/>
+      <c r="K147" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="148" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="10"/>
@@ -2472,7 +2907,10 @@
       <c r="H148" s="7"/>
       <c r="I148" s="7"/>
       <c r="J148" s="7"/>
-      <c r="K148" s="7"/>
+      <c r="K148" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="149" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="10"/>
@@ -2485,7 +2923,10 @@
       <c r="H149" s="7"/>
       <c r="I149" s="7"/>
       <c r="J149" s="7"/>
-      <c r="K149" s="7"/>
+      <c r="K149" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="150" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="10"/>
@@ -2498,7 +2939,10 @@
       <c r="H150" s="7"/>
       <c r="I150" s="7"/>
       <c r="J150" s="7"/>
-      <c r="K150" s="7"/>
+      <c r="K150" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="151" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="10"/>
@@ -2511,7 +2955,10 @@
       <c r="H151" s="7"/>
       <c r="I151" s="7"/>
       <c r="J151" s="7"/>
-      <c r="K151" s="7"/>
+      <c r="K151" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="152" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="10"/>
@@ -2524,7 +2971,10 @@
       <c r="H152" s="7"/>
       <c r="I152" s="7"/>
       <c r="J152" s="7"/>
-      <c r="K152" s="7"/>
+      <c r="K152" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="153" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="10"/>
@@ -2537,7 +2987,10 @@
       <c r="H153" s="7"/>
       <c r="I153" s="7"/>
       <c r="J153" s="7"/>
-      <c r="K153" s="7"/>
+      <c r="K153" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="154" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="10"/>
@@ -2550,7 +3003,10 @@
       <c r="H154" s="7"/>
       <c r="I154" s="7"/>
       <c r="J154" s="7"/>
-      <c r="K154" s="7"/>
+      <c r="K154" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="155" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="10"/>
@@ -2563,7 +3019,10 @@
       <c r="H155" s="7"/>
       <c r="I155" s="7"/>
       <c r="J155" s="7"/>
-      <c r="K155" s="7"/>
+      <c r="K155" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="156" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="10"/>
@@ -2576,7 +3035,10 @@
       <c r="H156" s="7"/>
       <c r="I156" s="7"/>
       <c r="J156" s="7"/>
-      <c r="K156" s="7"/>
+      <c r="K156" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="157" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="10"/>
@@ -2589,7 +3051,10 @@
       <c r="H157" s="7"/>
       <c r="I157" s="7"/>
       <c r="J157" s="7"/>
-      <c r="K157" s="7"/>
+      <c r="K157" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="158" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="10"/>
@@ -2602,7 +3067,10 @@
       <c r="H158" s="7"/>
       <c r="I158" s="7"/>
       <c r="J158" s="7"/>
-      <c r="K158" s="7"/>
+      <c r="K158" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="159" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="10"/>
@@ -2615,7 +3083,10 @@
       <c r="H159" s="7"/>
       <c r="I159" s="7"/>
       <c r="J159" s="7"/>
-      <c r="K159" s="7"/>
+      <c r="K159" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="160" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="10"/>
@@ -2628,7 +3099,10 @@
       <c r="H160" s="7"/>
       <c r="I160" s="7"/>
       <c r="J160" s="7"/>
-      <c r="K160" s="7"/>
+      <c r="K160" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="161" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="10"/>
@@ -2641,7 +3115,10 @@
       <c r="H161" s="7"/>
       <c r="I161" s="7"/>
       <c r="J161" s="7"/>
-      <c r="K161" s="7"/>
+      <c r="K161" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="162" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="10"/>
@@ -2654,7 +3131,10 @@
       <c r="H162" s="7"/>
       <c r="I162" s="7"/>
       <c r="J162" s="7"/>
-      <c r="K162" s="7"/>
+      <c r="K162" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="163" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="10"/>
@@ -2667,7 +3147,10 @@
       <c r="H163" s="7"/>
       <c r="I163" s="7"/>
       <c r="J163" s="7"/>
-      <c r="K163" s="7"/>
+      <c r="K163" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="164" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="10"/>
@@ -2680,7 +3163,10 @@
       <c r="H164" s="7"/>
       <c r="I164" s="7"/>
       <c r="J164" s="7"/>
-      <c r="K164" s="7"/>
+      <c r="K164" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="165" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="10"/>
@@ -2693,7 +3179,10 @@
       <c r="H165" s="7"/>
       <c r="I165" s="7"/>
       <c r="J165" s="7"/>
-      <c r="K165" s="7"/>
+      <c r="K165" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="166" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="10"/>
@@ -2706,7 +3195,10 @@
       <c r="H166" s="7"/>
       <c r="I166" s="7"/>
       <c r="J166" s="7"/>
-      <c r="K166" s="7"/>
+      <c r="K166" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="167" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="10"/>
@@ -2719,7 +3211,10 @@
       <c r="H167" s="7"/>
       <c r="I167" s="7"/>
       <c r="J167" s="7"/>
-      <c r="K167" s="7"/>
+      <c r="K167" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="168" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="10"/>
@@ -2732,7 +3227,10 @@
       <c r="H168" s="7"/>
       <c r="I168" s="7"/>
       <c r="J168" s="7"/>
-      <c r="K168" s="7"/>
+      <c r="K168" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="169" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="10"/>
@@ -2745,7 +3243,10 @@
       <c r="H169" s="7"/>
       <c r="I169" s="7"/>
       <c r="J169" s="7"/>
-      <c r="K169" s="7"/>
+      <c r="K169" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="170" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="10"/>
@@ -2758,7 +3259,10 @@
       <c r="H170" s="7"/>
       <c r="I170" s="7"/>
       <c r="J170" s="7"/>
-      <c r="K170" s="7"/>
+      <c r="K170" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="171" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="10"/>
@@ -2771,7 +3275,10 @@
       <c r="H171" s="7"/>
       <c r="I171" s="7"/>
       <c r="J171" s="7"/>
-      <c r="K171" s="7"/>
+      <c r="K171" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="172" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="10"/>
@@ -2784,7 +3291,10 @@
       <c r="H172" s="7"/>
       <c r="I172" s="7"/>
       <c r="J172" s="7"/>
-      <c r="K172" s="7"/>
+      <c r="K172" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="173" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="10"/>
@@ -2797,7 +3307,10 @@
       <c r="H173" s="7"/>
       <c r="I173" s="7"/>
       <c r="J173" s="7"/>
-      <c r="K173" s="7"/>
+      <c r="K173" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="174" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="10"/>
@@ -2810,7 +3323,10 @@
       <c r="H174" s="7"/>
       <c r="I174" s="7"/>
       <c r="J174" s="7"/>
-      <c r="K174" s="7"/>
+      <c r="K174" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="175" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="10"/>
@@ -2823,7 +3339,10 @@
       <c r="H175" s="7"/>
       <c r="I175" s="7"/>
       <c r="J175" s="7"/>
-      <c r="K175" s="7"/>
+      <c r="K175" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="176" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="10"/>
@@ -2836,7 +3355,10 @@
       <c r="H176" s="7"/>
       <c r="I176" s="7"/>
       <c r="J176" s="7"/>
-      <c r="K176" s="7"/>
+      <c r="K176" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="177" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="10"/>
@@ -2849,7 +3371,10 @@
       <c r="H177" s="7"/>
       <c r="I177" s="7"/>
       <c r="J177" s="7"/>
-      <c r="K177" s="7"/>
+      <c r="K177" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="178" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="10"/>
@@ -2862,7 +3387,10 @@
       <c r="H178" s="7"/>
       <c r="I178" s="7"/>
       <c r="J178" s="7"/>
-      <c r="K178" s="7"/>
+      <c r="K178" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="179" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="10"/>
@@ -2875,7 +3403,10 @@
       <c r="H179" s="7"/>
       <c r="I179" s="7"/>
       <c r="J179" s="7"/>
-      <c r="K179" s="7"/>
+      <c r="K179" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="180" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="10"/>
@@ -2888,7 +3419,10 @@
       <c r="H180" s="7"/>
       <c r="I180" s="7"/>
       <c r="J180" s="7"/>
-      <c r="K180" s="7"/>
+      <c r="K180" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="181" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="10"/>
@@ -2901,7 +3435,10 @@
       <c r="H181" s="7"/>
       <c r="I181" s="7"/>
       <c r="J181" s="7"/>
-      <c r="K181" s="7"/>
+      <c r="K181" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="182" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="10"/>
@@ -2914,7 +3451,10 @@
       <c r="H182" s="7"/>
       <c r="I182" s="7"/>
       <c r="J182" s="7"/>
-      <c r="K182" s="7"/>
+      <c r="K182" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="183" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="10"/>
@@ -2927,7 +3467,10 @@
       <c r="H183" s="7"/>
       <c r="I183" s="7"/>
       <c r="J183" s="7"/>
-      <c r="K183" s="7"/>
+      <c r="K183" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="184" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="10"/>
@@ -2940,7 +3483,10 @@
       <c r="H184" s="7"/>
       <c r="I184" s="7"/>
       <c r="J184" s="7"/>
-      <c r="K184" s="7"/>
+      <c r="K184" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="185" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="10"/>
@@ -2953,7 +3499,10 @@
       <c r="H185" s="7"/>
       <c r="I185" s="7"/>
       <c r="J185" s="7"/>
-      <c r="K185" s="7"/>
+      <c r="K185" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="186" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="10"/>
@@ -2966,7 +3515,10 @@
       <c r="H186" s="7"/>
       <c r="I186" s="7"/>
       <c r="J186" s="7"/>
-      <c r="K186" s="7"/>
+      <c r="K186" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="187" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="10"/>
@@ -2979,7 +3531,10 @@
       <c r="H187" s="7"/>
       <c r="I187" s="7"/>
       <c r="J187" s="7"/>
-      <c r="K187" s="7"/>
+      <c r="K187" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="188" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="10"/>
@@ -2992,7 +3547,10 @@
       <c r="H188" s="7"/>
       <c r="I188" s="7"/>
       <c r="J188" s="7"/>
-      <c r="K188" s="7"/>
+      <c r="K188" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="189" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A189" s="10"/>
@@ -3005,7 +3563,10 @@
       <c r="H189" s="7"/>
       <c r="I189" s="7"/>
       <c r="J189" s="7"/>
-      <c r="K189" s="7"/>
+      <c r="K189" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="190" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A190" s="10"/>
@@ -3018,7 +3579,10 @@
       <c r="H190" s="7"/>
       <c r="I190" s="7"/>
       <c r="J190" s="7"/>
-      <c r="K190" s="7"/>
+      <c r="K190" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="191" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="10"/>
@@ -3031,7 +3595,10 @@
       <c r="H191" s="7"/>
       <c r="I191" s="7"/>
       <c r="J191" s="7"/>
-      <c r="K191" s="7"/>
+      <c r="K191" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="192" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="10"/>
@@ -3044,7 +3611,10 @@
       <c r="H192" s="7"/>
       <c r="I192" s="7"/>
       <c r="J192" s="7"/>
-      <c r="K192" s="7"/>
+      <c r="K192" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="193" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="10"/>
@@ -3057,7 +3627,10 @@
       <c r="H193" s="7"/>
       <c r="I193" s="7"/>
       <c r="J193" s="7"/>
-      <c r="K193" s="7"/>
+      <c r="K193" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="194" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="10"/>
@@ -3070,7 +3643,10 @@
       <c r="H194" s="7"/>
       <c r="I194" s="7"/>
       <c r="J194" s="7"/>
-      <c r="K194" s="7"/>
+      <c r="K194" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="195" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="10"/>
@@ -3083,7 +3659,10 @@
       <c r="H195" s="7"/>
       <c r="I195" s="7"/>
       <c r="J195" s="7"/>
-      <c r="K195" s="7"/>
+      <c r="K195" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
     </row>
     <row r="196" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A196" s="10"/>
@@ -3096,7 +3675,10 @@
       <c r="H196" s="7"/>
       <c r="I196" s="7"/>
       <c r="J196" s="7"/>
-      <c r="K196" s="7"/>
+      <c r="K196" s="6" t="str">
+        <f t="shared" ref="K196:K259" si="3">IF(A196="","",SUM(D196:J196))</f>
+        <v/>
+      </c>
     </row>
     <row r="197" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="10"/>
@@ -3109,7 +3691,10 @@
       <c r="H197" s="7"/>
       <c r="I197" s="7"/>
       <c r="J197" s="7"/>
-      <c r="K197" s="7"/>
+      <c r="K197" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
     </row>
     <row r="198" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="10"/>
@@ -3122,7 +3707,10 @@
       <c r="H198" s="7"/>
       <c r="I198" s="7"/>
       <c r="J198" s="7"/>
-      <c r="K198" s="7"/>
+      <c r="K198" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
     </row>
     <row r="199" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="10"/>
@@ -3135,7 +3723,10 @@
       <c r="H199" s="7"/>
       <c r="I199" s="7"/>
       <c r="J199" s="7"/>
-      <c r="K199" s="7"/>
+      <c r="K199" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
     </row>
     <row r="200" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="10"/>
@@ -3148,7 +3739,1372 @@
       <c r="H200" s="7"/>
       <c r="I200" s="7"/>
       <c r="J200" s="7"/>
-      <c r="K200" s="7"/>
+      <c r="K200" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="201" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K201" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="202" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K202" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="203" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K203" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="204" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K204" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="205" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K205" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="206" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K206" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="207" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K207" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="208" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K208" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="209" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K209" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="210" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K210" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="211" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K211" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="212" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K212" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="213" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K213" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="214" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K214" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="215" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K215" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="216" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K216" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="217" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K217" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="218" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K218" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="219" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K219" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="220" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K220" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="221" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K221" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="222" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K222" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="223" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K223" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="224" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K224" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="225" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K225" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="226" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K226" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="227" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K227" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="228" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K228" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="229" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K229" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="230" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K230" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="231" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K231" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="232" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K232" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="233" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K233" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="234" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K234" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="235" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K235" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="236" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K236" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="237" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K237" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="238" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K238" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="239" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K239" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="240" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K240" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="241" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K241" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="242" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K242" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="243" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K243" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="244" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K244" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="245" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K245" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="246" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K246" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="247" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K247" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="248" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K248" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="249" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K249" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="250" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K250" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="251" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K251" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="252" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K252" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="253" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K253" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="254" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K254" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="255" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K255" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="256" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K256" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="257" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K257" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="258" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K258" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="259" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K259" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="260" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K260" s="6" t="str">
+        <f t="shared" ref="K260:K323" si="4">IF(A260="","",SUM(D260:J260))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="261" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K261" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="262" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K262" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="263" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K263" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="264" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K264" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="265" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K265" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="266" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K266" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="267" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K267" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="268" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K268" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="269" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K269" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="270" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K270" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="271" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K271" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="272" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K272" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="273" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K273" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="274" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K274" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="275" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K275" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="276" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K276" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="277" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K277" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="278" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K278" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="279" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K279" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="280" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K280" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="281" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K281" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="282" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K282" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="283" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K283" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="284" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K284" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="285" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K285" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="286" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K286" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="287" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K287" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="288" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K288" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="289" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K289" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="290" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K290" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="291" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K291" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="292" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K292" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="293" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K293" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="294" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K294" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="295" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K295" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="296" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K296" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="297" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K297" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="298" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K298" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="299" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K299" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="300" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K300" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="301" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K301" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="302" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K302" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="303" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K303" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="304" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K304" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="305" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K305" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="306" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K306" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="307" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K307" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="308" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K308" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="309" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K309" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="310" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K310" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="311" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K311" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="312" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K312" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="313" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K313" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="314" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K314" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="315" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K315" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="316" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K316" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="317" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K317" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="318" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K318" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="319" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K319" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="320" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K320" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="321" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K321" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="322" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K322" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="323" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K323" s="6" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="324" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K324" s="6" t="str">
+        <f t="shared" ref="K324:K387" si="5">IF(A324="","",SUM(D324:J324))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="325" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K325" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="326" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K326" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="327" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K327" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="328" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K328" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="329" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K329" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="330" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K330" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="331" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K331" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="332" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K332" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="333" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K333" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="334" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K334" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="335" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K335" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="336" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K336" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="337" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K337" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="338" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K338" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="339" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K339" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="340" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K340" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="341" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K341" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="342" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K342" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="343" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K343" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="344" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K344" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="345" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K345" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="346" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K346" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="347" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K347" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="348" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K348" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="349" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K349" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="350" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K350" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="351" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K351" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="352" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K352" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="353" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K353" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="354" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K354" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="355" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K355" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="356" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K356" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="357" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K357" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="358" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K358" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="359" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K359" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="360" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K360" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="361" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K361" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="362" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K362" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="363" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K363" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="364" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K364" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="365" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K365" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="366" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K366" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="367" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K367" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="368" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K368" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="369" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K369" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="370" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K370" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="371" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K371" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="372" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K372" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="373" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K373" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="374" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K374" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="375" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K375" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="376" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K376" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="377" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K377" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="378" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K378" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="379" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K379" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="380" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K380" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="381" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K381" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="382" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K382" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="383" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K383" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="384" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K384" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="385" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K385" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="386" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K386" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="387" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K387" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="388" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K388" s="6" t="str">
+        <f t="shared" ref="K388:K427" si="6">IF(A388="","",SUM(D388:J388))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="389" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K389" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="390" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K390" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="391" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K391" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="392" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K392" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="393" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K393" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="394" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K394" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="395" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K395" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="396" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K396" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="397" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K397" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="398" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K398" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="399" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K399" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="400" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K400" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="401" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K401" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="402" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K402" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="403" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K403" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="404" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K404" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="405" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K405" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="406" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K406" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="407" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K407" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="408" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K408" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="409" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K409" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="410" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K410" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="411" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K411" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="412" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K412" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="413" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K413" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="414" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K414" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="415" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K415" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="416" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K416" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="417" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K417" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="418" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K418" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="419" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K419" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="420" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K420" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="421" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K421" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="422" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K422" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="423" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K423" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="424" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K424" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="425" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K425" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="426" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K426" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="427" spans="11:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K427" s="6" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>